<commit_message>
Cobertura de todas as classes
</commit_message>
<xml_diff>
--- a/tabelas_classes_excel/Tabela_3-11_O_Guerreiro.xlsx
+++ b/tabelas_classes_excel/Tabela_3-11_O_Guerreiro.xlsx
@@ -764,9 +764,6 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -960,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1013,31 +1010,6 @@
           <t>C7</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>C8</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>C10</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>C11</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>C12</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1715,685 +1687,6 @@
       <c r="F23" t="inlineStr">
         <is>
           <t>Talento Adicional</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Características da Classe</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Arco Curto (1d6, dec.x 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Usar Armas e Armaduras: Um guerreiro sabe usar todas as armas simples</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Seleção de Perícias: Esc</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>e comuns, armaduras (leves, médias e pesadas) e escudos (incluindo escudos de</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>a 3 + modificador de Inteligê</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>corpo).</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Talento: Foco em Arma (e</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Talentos Adicionais: No 1* nível, um guerreiro recebe um talento adicional</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Talento Adicional (Guerr</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>relacionado ao combate, além do talento normal concedido aos demais personagens</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Personagens com Força 12 ou i</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>de 1° nível e o talento adicional fornecido aos humanos. O guerreiro recebe um</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Talento Adicional (human</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>talento adicional no 2° nível e a cada dois níveis subseqüentes (4°, 6°, 8°, 10°, 12°,</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Equipamento: Mochila com</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>14°, 16°, 18° e 20°). Esses talentos adicionais precisam ser selecionados da lista de</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>saco, pederneira e isqueiro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>talentos adicionais do guerreiro, na Tabela 5-1: Talentos. Um guerreiro ainda precisa</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Dinheiro: 2d4 PO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>atender aos pré-requisitos para escolher um talento adicional, inclusive valores de</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Perícia</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Gr</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>habilidade ou bônus base de ataque mínimo (veja as descrições e pré-requisitos dos</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>talentos no Capítulo 5).</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Natação</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Esses talentos são adicionados ao talento que um personagem de qualquer classe</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Observar (oc)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>receberá a cada três níveis (consulte a Tabela 3-2: Benefícios e Experiência Conforme</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Ouvir (oc)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>o Nível). Para selecionar esses últimos, o guerreiro não precisa se limitar à relação</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Saltar</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>de talentos adicionais do guerreiro.</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Cavalgar</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Escalar</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Conjunto Inicial para Guerreiro Anão</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Armadura: Brunea (+4 CA, -4 de penalidade de armadura, 6 m de desloca-</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Intimidação</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>mento, 15 kg).</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Procurar (oc)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Escudo grande de madeira (+2 CA, -2 de penalidade de armadura)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Armas: Machado de guerra anão (1d10, dec.x 3, 4 kg, uma mão, cortante).</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Arco Curto (1d6, dec.x 3,18 m, 1 kg, perfurante)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Seleção de Perícias: Escolha uma quantidade de graduações de perícias igual</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>a 2 + modificador de Inteligência.</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Os ladinos têm pouco em</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>são charlatões habilidosos. O</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Perícia</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Graduações</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Habilidade</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Armadura</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>criminosos. A única coisa em</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Cavalgar</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Des</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>de recursos. Em geral, os lad</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>alvos menos desejam: invadir</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Escalar</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>For</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>-6</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>letal em segurança, obter pla</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Intimidação</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Car</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>guarda ou retirar o dinheiro</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Natação</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>For</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>-12</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Aventuras: Os ladinos s</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Observar (oc)</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Sab</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>os seus atos: conseguir o que</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Ouvir (oc)</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Sab</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Alguns procuram fama, infâmia</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>uma armadilha ou não disparar</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Procurar (oc)</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Int</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ladinos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Saltar</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>For</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>-6</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Características: Os lad</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>desenvolvimento de qualquer v</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Talento: Foco em Arma (machado de guerra anão)</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>aos membros de outras classes</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Talento Adicional (Guerreiro): Personagens com Força 13+: Ataque Poderoso;</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>precisos e infligir enormes q</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Personagens com Força 12 ou inferior: Iniciativa Aprimorada.</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Eles possuem um sexto s</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Equipamento: Mochila com cantil, um dia de rações de viagem, saco de dormir,</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>do sigilo, a evasão e os ataq</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>saco, pederneira e isqueiro. Aljava com 20 flechas.</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>e poderes quase místicos. Alé</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Dinheiro: 4d4 PO.</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>os ladinos podem “fingir” o s</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>e usar quase todos os itens m</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Conjunto Inicial para Humano Guerreiro</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Tendência: Os ladinos s</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Armadura: Brunea (+4 CA, -4 de penalidade de armadura, 6 m de desloca-</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>que sejam Caóticos em vez de</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>mento, 15 kg).</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>qualquer tendência.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Armas: Espada larga (2d6, dec. 19-20/x2,4 kg, duas mãos, cortante).</t>
         </is>
       </c>
     </row>

</xml_diff>